<commit_message>
Save local changes before rebase
</commit_message>
<xml_diff>
--- a/health_reports.xlsx
+++ b/health_reports.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -693,10 +693,8 @@
       <c r="B10" t="n">
         <v>25</v>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>354787</t>
-        </is>
+      <c r="C10" t="n">
+        <v>354787</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -711,6 +709,36 @@
       <c r="F10" t="inlineStr">
         <is>
           <t>fdgfvb</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>sdfds</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>25</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>9876543212</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>['Stomach Pain']</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>dfdbvcbt</t>
         </is>
       </c>
     </row>

</xml_diff>